<commit_message>
feat: GM panel autocomplete and current updates
</commit_message>
<xml_diff>
--- a/tables/datas/item/#Item-道具系统表.xlsx
+++ b/tables/datas/item/#Item-道具系统表.xlsx
@@ -715,6 +715,11 @@
       <c r="G5" t="n">
         <v>0</v>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>item_1001_xianbei.png</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>恢复少量生命值</t>
@@ -767,7 +772,6 @@
       <c r="L6" t="n">
         <v>2</v>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>0</v>
       </c>

</xml_diff>

<commit_message>
feat: text inventory panel (backpack)
</commit_message>
<xml_diff>
--- a/tables/datas/item/#Item-道具系统表.xlsx
+++ b/tables/datas/item/#Item-道具系统表.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R7"/>
+  <dimension ref="A1:R21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,7 +767,6 @@
       <c r="L6" t="n">
         <v>2</v>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>0</v>
       </c>
@@ -821,6 +820,648 @@
       <c r="P7" t="b">
         <v>0</v>
       </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="n">
+        <v>1003</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>药草</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n">
+        <v>403</v>
+      </c>
+      <c r="F8" t="n">
+        <v>99</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>恢复少量生命值</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>30</v>
+      </c>
+      <c r="O8" t="n">
+        <v>5</v>
+      </c>
+      <c r="P8" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="B9" t="n">
+        <v>1004</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>铁剑</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n">
+        <v>421</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>近战武器</t>
+        </is>
+      </c>
+      <c r="L9" t="n">
+        <v>5</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>100</v>
+      </c>
+      <c r="P9" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="B10" t="n">
+        <v>1005</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>精灵之弓</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n">
+        <v>422</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>远程武器</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" t="n">
+        <v>300</v>
+      </c>
+      <c r="P10" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="B11" t="n">
+        <v>1006</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>龙鳞铠甲</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>220</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>厚重护甲</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>7</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>800</v>
+      </c>
+      <c r="P11" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="B12" t="n">
+        <v>1007</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>传说级法杖</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" t="n">
+        <v>423</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>4</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>蕴含强大魔力</t>
+        </is>
+      </c>
+      <c r="L12" t="n">
+        <v>8</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" t="n">
+        <v>2000</v>
+      </c>
+      <c r="P12" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="B13" t="n">
+        <v>1008</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>小型生命药水</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" t="n">
+        <v>403</v>
+      </c>
+      <c r="F13" t="n">
+        <v>99</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>恢复生命值</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>9</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>heal</t>
+        </is>
+      </c>
+      <c r="N13" t="n">
+        <v>80</v>
+      </c>
+      <c r="O13" t="n">
+        <v>15</v>
+      </c>
+      <c r="P13" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="B14" t="n">
+        <v>1009</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>高级魔法卷轴</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n">
+        <v>403</v>
+      </c>
+      <c r="F14" t="n">
+        <v>50</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>记载高级法术</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>10</v>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
+        <v>250</v>
+      </c>
+      <c r="P14" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="B15" t="n">
+        <v>1010</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>普通矿石</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>11</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1101</v>
+      </c>
+      <c r="F15" t="n">
+        <v>99</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>常见锻造材料</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>11</v>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" t="n">
+        <v>8</v>
+      </c>
+      <c r="P15" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="B16" t="n">
+        <v>1011</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>秘银锭</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>11</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1101</v>
+      </c>
+      <c r="F16" t="n">
+        <v>99</v>
+      </c>
+      <c r="G16" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>珍贵金属材料</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>12</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>120</v>
+      </c>
+      <c r="P16" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="B17" t="n">
+        <v>1012</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>龙之逆鳞</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>11</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1101</v>
+      </c>
+      <c r="F17" t="n">
+        <v>10</v>
+      </c>
+      <c r="G17" t="n">
+        <v>3</v>
+      </c>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>稀有锻造材料</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>13</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" t="n">
+        <v>1500</v>
+      </c>
+      <c r="P17" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="B18" t="n">
+        <v>1013</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>古代金币</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="n">
+        <v>102</v>
+      </c>
+      <c r="F18" t="n">
+        <v>999</v>
+      </c>
+      <c r="G18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>古代流通货币</t>
+        </is>
+      </c>
+      <c r="L18" t="n">
+        <v>14</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>add_gold</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>500</v>
+      </c>
+      <c r="O18" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="B19" t="n">
+        <v>1014</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>勇者徽章</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>6</v>
+      </c>
+      <c r="E19" t="n">
+        <v>601</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>证明勇气的徽章</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>15</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="B20" t="n">
+        <v>1015</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>普通钥匙</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>5</v>
+      </c>
+      <c r="E20" t="n">
+        <v>502</v>
+      </c>
+      <c r="F20" t="n">
+        <v>20</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>开启普通宝箱</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>16</v>
+      </c>
+      <c r="M20" t="inlineStr"/>
+      <c r="N20" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" t="n">
+        <v>50</v>
+      </c>
+      <c r="P20" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="B21" t="n">
+        <v>1016</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>神秘宝箱</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>5</v>
+      </c>
+      <c r="E21" t="n">
+        <v>501</v>
+      </c>
+      <c r="F21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>装有神秘物品</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>17</v>
+      </c>
+      <c r="M21" t="inlineStr"/>
+      <c r="N21" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" t="n">
+        <v>300</v>
+      </c>
+      <c r="P21" t="b">
+        <v>1</v>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>